<commit_message>
Add 'How It Works' tab and expand notes in verification sheet
Adds a second sheet ('How It Works') with plain-English explanations of
every calculation step: how YTD taxable income is inferred when left
blank, why the 0.9235 SE factor exists, how LTCG stacking works, what
safe harbor means, the order credits are applied, etc.

Also expands column C notes throughout the Verify 2025 sheet so each
row explains what number to enter and where to find it on your paystub
or tax documents.

https://claude.ai/code/session_01Y7YPpxMuoBgeSrJ7JB9ZH7
</commit_message>
<xml_diff>
--- a/tax-withholding-estimator/examples/tax_verify_2025.xlsx
+++ b/tax-withholding-estimator/examples/tax_verify_2025.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Verify 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How It Works" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +62,13 @@
       <color rgb="00546E7A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004A148C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +108,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -146,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -193,6 +204,13 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -564,7 +582,7 @@
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -578,7 +596,7 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells = user inputs.  Blue = Excel formula.  Green = final results.  Paste twe output in column D to compare.</t>
+          <t>Yellow = input you type.  Blue = Excel formula.  Green = key result.  See the 'How It Works' tab for plain-English logic explanations.</t>
         </is>
       </c>
     </row>
@@ -650,7 +668,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Update if using a different filing status or age-65/blind add-on</t>
+          <t>Single $15K | MFJ $30K | HoH $22.5K | MFS $15K  (+$2K if 65+/blind, single)</t>
         </is>
       </c>
     </row>
@@ -712,7 +730,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Box 1 equivalent on your stub</t>
+          <t>Gross pay MINUS pre-tax deductions (401k, HSA, etc.) — your 'Federal Taxable' line</t>
         </is>
       </c>
     </row>
@@ -725,7 +743,11 @@
       <c r="B15" s="10" t="n">
         <v>410</v>
       </c>
-      <c r="C15" s="8" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>'Federal Income Tax' on your paystub — NOT SS or Medicare</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -736,7 +758,11 @@
       <c r="B16" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="C16" s="8" t="inlineStr"/>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Count paychecks left this calendar year including the next one</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -749,7 +775,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Leave 0 to infer from per-period amount</t>
+          <t>From paystub YTD column. Leave 0 → inferred as elapsed×per-period (see How It Works tab)</t>
         </is>
       </c>
     </row>
@@ -762,7 +788,11 @@
       <c r="B18" s="10" t="n">
         <v>4920</v>
       </c>
-      <c r="C18" s="8" t="inlineStr"/>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>From paystub YTD column. Leave 0 → inferred as elapsed×per-period</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="6" customHeight="1">
       <c r="A19" s="11" t="n"/>
@@ -788,7 +818,11 @@
       <c r="B21" s="10" t="n">
         <v>350</v>
       </c>
-      <c r="C21" s="8" t="inlineStr"/>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>1099-INT box 1</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -799,7 +833,11 @@
       <c r="B22" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="C22" s="8" t="inlineStr"/>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>1099-DIV box 1a</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -812,7 +850,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Must be ≤ ordinary dividends; part of LTCG rate pool</t>
+          <t>1099-DIV box 1b — must be ≤ ordinary dividends; taxed at 0/15/20% (see How It Works)</t>
         </is>
       </c>
     </row>
@@ -825,7 +863,11 @@
       <c r="B24" s="10" t="n">
         <v>5000</v>
       </c>
-      <c r="C24" s="8" t="inlineStr"/>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>1099-R box 2a taxable amount — Roth conversions, traditional withdrawals</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -836,7 +878,11 @@
       <c r="B25" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="C25" s="8" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Held &gt;1 year; taxed at 0/15/20% stacked on top of ordinary income (see How It Works)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -847,7 +893,11 @@
       <c r="B26" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="8" t="inlineStr"/>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Held ≤1 year; taxed as ordinary income</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -858,7 +908,11 @@
       <c r="B27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="8" t="inlineStr"/>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Schedule C profit (after business expenses). SE tax computed in Section ⑦</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -912,7 +966,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Adjustments (above-the-line)</t>
+          <t xml:space="preserve">  Adjustments (above-the-line — reduce income before deduction)</t>
         </is>
       </c>
       <c r="B33" s="5" t="n"/>
@@ -928,7 +982,11 @@
       <c r="B34" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C34" s="8" t="inlineStr"/>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Deductible if no workplace plan, or income below phaseout; up to $7,000 ($8K age 50+)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
@@ -939,7 +997,11 @@
       <c r="B35" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="C35" s="8" t="inlineStr"/>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Employee-paid HSA contributions not via payroll; 2025 limit $4,300 self / $8,550 family</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -950,7 +1012,11 @@
       <c r="B36" s="10" t="n">
         <v>1200</v>
       </c>
-      <c r="C36" s="8" t="inlineStr"/>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Deductible up to $2,500; phases out at $85K–$100K AGI (single 2025)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
@@ -961,7 +1027,11 @@
       <c r="B37" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C37" s="8" t="inlineStr"/>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Educator expenses ($300), alimony (pre-2019 divorces), self-employed health ins., etc.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="6" customHeight="1">
       <c r="A38" s="11" t="n"/>
@@ -989,7 +1059,7 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>0 → uses standard deduction</t>
+          <t>Mortgage int + state/local taxes (cap $10K) + charity + medical &gt;7.5% AGI. 0 → standard wins</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1072,11 @@
       <c r="B41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C41" s="8" t="inlineStr"/>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Up to $2,000/child under 17; phases out above $200K AGI (single). Enter expected credit amount.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
@@ -1013,7 +1087,11 @@
       <c r="B42" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C42" s="8" t="inlineStr"/>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Education credits, child/dependent care, savers credit, etc. Cannot exceed tax owed.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
@@ -1024,7 +1102,11 @@
       <c r="B43" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C43" s="8" t="inlineStr"/>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>EITC, Additional Child Tax Credit, American Opportunity Credit (40% refundable). Can produce refund.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="6" customHeight="1">
       <c r="A44" s="11" t="n"/>
@@ -1050,7 +1132,11 @@
       <c r="B46" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C46" s="8" t="inlineStr"/>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Quarterly Form 1040-ES payments already made this year</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
@@ -1061,7 +1147,11 @@
       <c r="B47" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C47" s="8" t="inlineStr"/>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Backup withholding, pension withholding, etc.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
@@ -1072,7 +1162,11 @@
       <c r="B48" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C48" s="8" t="inlineStr"/>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Positive = over-withhold to get a refund. Negative = accept owing up to this amount at filing.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -1085,7 +1179,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>For safe-harbor calculation</t>
+          <t>Your actual 2024 total tax (Form 1040 line 24). Used for safe-harbor calculation in Section ⑪</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1192,11 @@
       <c r="B50" s="10" t="n">
         <v>71000</v>
       </c>
-      <c r="C50" s="8" t="inlineStr"/>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>2024 AGI (Form 1040 line 11). If &gt;$150K, safe harbor requires 110% of prior-year tax.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="6" customHeight="1">
       <c r="A51" s="11" t="n"/>
@@ -1125,10 +1223,9 @@
         <f>$B$13-$B$16</f>
         <v/>
       </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>periods_per_year − remaining</t>
-        </is>
+      <c r="C53" s="8">
+        <f> periods_per_year − remaining. Example: biweekly 26 total, 14 remaining → 12 elapsed</f>
+        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -1143,21 +1240,24 @@
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>From input if provided, else inferred</t>
+          <t>Uses input if non-zero; otherwise infers as elapsed×per-period. Enter actual YTD from paystub for accuracy.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>Projected taxable wages</t>
+          <t>Projected full-year taxable wages</t>
         </is>
       </c>
       <c r="B55" s="13">
         <f>$B$54+$B$14*$B$16</f>
         <v/>
       </c>
-      <c r="C55" s="8" t="inlineStr"/>
+      <c r="C55" s="8">
+        <f> YTD used + (remaining × per-period). Best estimate of W-2 Box 1.</f>
+        <v/>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -1169,19 +1269,27 @@
         <f>IF($B$18&gt;0, $B$18, $B$15*$B$53)</f>
         <v/>
       </c>
-      <c r="C56" s="8" t="inlineStr"/>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Uses input if non-zero; otherwise infers as elapsed×per-period</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>Projected total withholding (job 1)</t>
+          <t>Projected total withholding (job 1 only)</t>
         </is>
       </c>
       <c r="B57" s="13">
         <f>$B$56+$B$15*$B$16</f>
         <v/>
       </c>
-      <c r="C57" s="8" t="inlineStr"/>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Projected if nothing changes. Add spouse/other withholding in Section ⑩.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
@@ -1193,7 +1301,11 @@
         <f>$B$55+$B$21+$B$22+$B$24+$B$26+$B$25+$B$27+$B$28+$B$29+$B$30</f>
         <v/>
       </c>
-      <c r="C58" s="8" t="inlineStr"/>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Sum of all income sources before any deductions or adjustments</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="6" customHeight="1">
       <c r="A59" s="11" t="n"/>
@@ -1213,7 +1325,7 @@
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>One-half SE tax deduction</t>
+          <t>One-half SE tax deduction (approx.)</t>
         </is>
       </c>
       <c r="B61" s="13">
@@ -1222,21 +1334,25 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Approx — exact calc in SE Tax section below; use that value</t>
+          <t>Quick estimate used here. Compare to exact value in Section ⑦ — they should agree. Large SE income? Update AGI manually.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>Total adjustments</t>
+          <t>Total adjustments (above-the-line)</t>
         </is>
       </c>
       <c r="B62" s="13">
         <f>$B$34+$B$35+$B$36+$B$37+$B$61</f>
         <v/>
       </c>
-      <c r="C62" s="8" t="inlineStr"/>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>IRA + HSA + student loan interest + other + ½ SE tax</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="14" t="inlineStr">
@@ -1248,7 +1364,11 @@
         <f>MAX(0, $B$58-$B$62)</f>
         <v/>
       </c>
-      <c r="C63" s="8" t="inlineStr"/>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Total income minus above-the-line adjustments. Many credits and phaseouts are based on AGI.</t>
+        </is>
+      </c>
       <c r="D63" s="16" t="n"/>
     </row>
     <row r="64" ht="6" customHeight="1">
@@ -1269,7 +1389,7 @@
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Deduction used (larger of standard/itemized)</t>
+          <t>Deduction used (larger of standard / itemized)</t>
         </is>
       </c>
       <c r="B66" s="13">
@@ -1278,7 +1398,7 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Standard = $15,000 for single 2025; update std_ded input for other status</t>
+          <t>Itemized wins only if it exceeds standard. Most filers use standard after 2017 TCJA.</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1412,10 @@
         <f>MAX(0, $B$63-$B$66)</f>
         <v/>
       </c>
-      <c r="C67" s="8" t="inlineStr"/>
+      <c r="C67" s="8">
+        <f> AGI − deduction. Brackets are applied to this number (after separating LTCG below).</f>
+        <v/>
+      </c>
       <c r="D67" s="16" t="n"/>
     </row>
     <row r="68" ht="6" customHeight="1">
@@ -1322,7 +1445,7 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Taxed at 0/15/20% rates — subtracted from ordinary TI</t>
+          <t>Removed from ordinary TI and taxed at 0/15/20% in Section ⑥. Capped at taxable income.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1459,10 @@
         <f>MAX(0, $B$67-$B$70)</f>
         <v/>
       </c>
-      <c r="C71" s="8" t="inlineStr"/>
+      <c r="C71" s="8">
+        <f> Taxable income − preferential. This is what the 10–37% brackets apply to.</f>
+        <v/>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
@@ -1350,7 +1476,7 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>IFS brackets: 10/12/22/24/32/35/37%  (2025 single)</t>
+          <t>Cumulative bracket amounts encoded: $1,192.50 at $11,925 / $5,578.50 at $48,475 / etc.</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1490,11 @@
         <f>IFS($B$71&lt;=0, 0.10, $B$71&lt;=11925, 0.10, $B$71&lt;=48475, 0.12, $B$71&lt;=103350, 0.22, $B$71&lt;=197300, 0.24, $B$71&lt;=250525, 0.32, $B$71&lt;=626350, 0.35, TRUE, 0.37)</f>
         <v/>
       </c>
-      <c r="C73" s="8" t="inlineStr"/>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>The rate that applies to your next dollar of ordinary income.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="6" customHeight="1">
       <c r="A74" s="11" t="n"/>
@@ -1384,7 +1514,7 @@
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>Room in 0% bracket</t>
+          <t>Room remaining in 0% bracket</t>
         </is>
       </c>
       <c r="B76" s="13">
@@ -1393,7 +1523,7 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>2025 single 0% LTCG threshold: $48,350</t>
+          <t>0% rate applies up to $48,350 of total TI (single 2025). Ordinary income fills this bucket first.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1537,11 @@
         <f>MIN($B$70, $B$76)</f>
         <v/>
       </c>
-      <c r="C77" s="8" t="inlineStr"/>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>The slice of preferential income that fits in the remaining 0% room.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
@@ -1419,7 +1553,11 @@
         <f>MAX(0, $B$70-$B$77)</f>
         <v/>
       </c>
-      <c r="C78" s="8" t="inlineStr"/>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>Spills into 15% or 20% bracket.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
@@ -1433,7 +1571,7 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>2025 single 15% LTCG threshold: $533,400</t>
+          <t>15% rate applies from $48,350 to $533,400 of total TI (single 2025).</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1597,11 @@
         <f>MAX(0, $B$78-$B$80)</f>
         <v/>
       </c>
-      <c r="C81" s="8" t="inlineStr"/>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Any preferential income above $533,400 total TI.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
@@ -1471,7 +1613,11 @@
         <f>$B$80*0.15+$B$81*0.20</f>
         <v/>
       </c>
-      <c r="C82" s="8" t="inlineStr"/>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>0% amount is free — no tax on that slice.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="6" customHeight="1">
       <c r="A83" s="11" t="n"/>
@@ -1491,31 +1637,39 @@
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>SE net earnings (×0.9235)</t>
+          <t>SE net earnings (× 0.9235 factor)</t>
         </is>
       </c>
       <c r="B85" s="13">
         <f>IF($B$27&lt;=0, 0, $B$27*0.9235)</f>
         <v/>
       </c>
-      <c r="C85" s="8" t="inlineStr"/>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>0.9235 = 1 − 0.0765 adjusts for the employer-half SS/Medicare that employees don't pay. See How It Works.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>SS wage base room (2025: $176,100)</t>
+          <t>Remaining SS wage base room (2025: $176,100)</t>
         </is>
       </c>
       <c r="B86" s="13">
         <f>MAX(0, 176100-$B$55-$B$30)</f>
         <v/>
       </c>
-      <c r="C86" s="8" t="inlineStr"/>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>SS tax only applies to earnings up to $176,100. If wages already exceed this, SE income has no SS portion.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>SE income subject to SS</t>
+          <t>SE net earnings subject to SS (12.4%)</t>
         </is>
       </c>
       <c r="B87" s="13">
@@ -1534,12 +1688,16 @@
         <f>IF($B$27&lt;=0, 0, $B$87*0.124 + $B$85*0.029)</f>
         <v/>
       </c>
-      <c r="C88" s="8" t="inlineStr"/>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Both halves (employee + employer equivalent) are owed by self-employed filers.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>One-half SE tax (above-the-line deduction)</t>
+          <t>One-half SE tax (exact above-the-line deduction)</t>
         </is>
       </c>
       <c r="B89" s="13">
@@ -1548,7 +1706,7 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>This is the exact value; the approximation above in Section ③ is close but update AGI if SE income is large</t>
+          <t>Deduct this amount above-the-line. Compare to the approx. in Section ③ — if different, update AGI manually.</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1735,11 @@
         <f>$B$55+$B$30+$B$85</f>
         <v/>
       </c>
-      <c r="C92" s="8" t="inlineStr"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>The base for Additional Medicare Tax. Your employer only sees their own wages — they miss spouse or SE income.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
@@ -1589,7 +1751,11 @@
         <f>MAX(0, $B$92-200000)*0.009</f>
         <v/>
       </c>
-      <c r="C93" s="8" t="inlineStr"/>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>Threshold: $200K single | $250K MFJ | $125K MFS. No SS component — Medicare only.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
@@ -1601,7 +1767,11 @@
         <f>MAX(0, $B$21+$B$22+$B$26+$B$25)</f>
         <v/>
       </c>
-      <c r="C94" s="8" t="inlineStr"/>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Interest + dividends + capital gains (short &amp; long). Does NOT include wages or SE income.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
@@ -1613,7 +1783,10 @@
         <f>MIN($B$94, MAX(0,$B$63-200000))*0.038</f>
         <v/>
       </c>
-      <c r="C95" s="8" t="inlineStr"/>
+      <c r="C95" s="8">
+        <f> 3.8% × MIN(net investment income, MAX(0, AGI − $200K)). Zero if AGI ≤ $200K.</f>
+        <v/>
+      </c>
     </row>
     <row r="96" ht="6" customHeight="1">
       <c r="A96" s="11" t="n"/>
@@ -1640,7 +1813,11 @@
         <f>$B$72+$B$82</f>
         <v/>
       </c>
-      <c r="C98" s="8" t="inlineStr"/>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Ordinary income tax + capital gains tax</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
@@ -1652,7 +1829,11 @@
         <f>$B$98+$B$88+$B$93+$B$95</f>
         <v/>
       </c>
-      <c r="C99" s="8" t="inlineStr"/>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Income tax + SE tax + Additional Medicare Tax + NIIT</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
@@ -1664,7 +1845,11 @@
         <f>MIN($B$41+$B$42, $B$99)</f>
         <v/>
       </c>
-      <c r="C100" s="8" t="inlineStr"/>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Capped at tax before credits — cannot go below $0. Refundable credits applied separately below.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="14" t="inlineStr">
@@ -1676,20 +1861,27 @@
         <f>MAX(0, $B$99-$B$100-$B$43)</f>
         <v/>
       </c>
-      <c r="C101" s="8" t="inlineStr"/>
+      <c r="C101" s="8">
+        <f> Tax before credits − nonrefundable credits − refundable credits. Cannot go below $0.</f>
+        <v/>
+      </c>
       <c r="D101" s="16" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>Effective rate</t>
+          <t>Effective tax rate</t>
         </is>
       </c>
       <c r="B102" s="17">
         <f>IF($B$63&gt;0, $B$101/$B$63, 0)</f>
         <v/>
       </c>
-      <c r="C102" s="8" t="inlineStr"/>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>Total liability ÷ AGI. Different from marginal rate — shows average tax burden.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="6" customHeight="1">
       <c r="A103" s="11" t="n"/>
@@ -1709,26 +1901,34 @@
     <row r="105" ht="15" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>Other payments (estimated tax + other withholding)</t>
+          <t>Other payments (estimated tax + withholding)</t>
         </is>
       </c>
       <c r="B105" s="13">
         <f>$B$46+$B$47+$B$31</f>
         <v/>
       </c>
-      <c r="C105" s="8" t="inlineStr"/>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Quarterly estimated tax payments + any other withholding sources + spouse withholding</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>Already secured (YTD withholding + other payments)</t>
+          <t>Already secured toward liability</t>
         </is>
       </c>
       <c r="B106" s="13">
         <f>$B$56+$B$105</f>
         <v/>
       </c>
-      <c r="C106" s="8" t="inlineStr"/>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>YTD withholding + all other payments. These are locked in — only future paychecks are adjustable.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
@@ -1742,21 +1942,24 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>0 for single-job; add other jobs' remaining withholding here</t>
+          <t>If you have a second job, enter its expected remaining withholding here so we don't double-count.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Required from remaining paychecks</t>
+          <t>Still needed from remaining paychecks</t>
         </is>
       </c>
       <c r="B108" s="13">
         <f>MAX(0, ($B$101+$B$48)-$B$106-$B$107)</f>
         <v/>
       </c>
-      <c r="C108" s="8" t="inlineStr"/>
+      <c r="C108" s="8">
+        <f> (Liability + target refund) − already secured − other future. This is the total gap.</f>
+        <v/>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="14" t="inlineStr">
@@ -1768,20 +1971,26 @@
         <f>IF($B$16&gt;0, $B$108/$B$16, 0)</f>
         <v/>
       </c>
-      <c r="C109" s="8" t="inlineStr"/>
+      <c r="C109" s="8">
+        <f> gap ÷ remaining periods. Set your W-4 so each check withholds at least this amount.</f>
+        <v/>
+      </c>
       <c r="D109" s="16" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>Additional withholding per paycheck (W-4 line 4c)</t>
+          <t>Extra per paycheck needed (W-4 line 4c)</t>
         </is>
       </c>
       <c r="B110" s="15">
         <f>MAX(0, $B$109-$B$15)</f>
         <v/>
       </c>
-      <c r="C110" s="8" t="inlineStr"/>
+      <c r="C110" s="8">
+        <f> recommended − current withholding per period. Enter this on Form W-4 Step 4(c) as extra withholding.</f>
+        <v/>
+      </c>
       <c r="D110" s="16" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1">
@@ -1794,7 +2003,11 @@
         <f>$B$57+$B$105-$B$101</f>
         <v/>
       </c>
-      <c r="C111" s="8" t="inlineStr"/>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>If you change NOTHING on your W-4. Positive = refund, negative = balance due at filing.</t>
+        </is>
+      </c>
       <c r="D111" s="16" t="n"/>
     </row>
     <row r="112" ht="6" customHeight="1">
@@ -1805,7 +2018,7 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>⑪ SAFE HARBOR  (penalty avoidance)</t>
+          <t>⑪ SAFE HARBOR  (minimum to avoid underpayment penalty)</t>
         </is>
       </c>
       <c r="B113" s="5" t="n"/>
@@ -1822,7 +2035,11 @@
         <f>$B$101*0.90</f>
         <v/>
       </c>
-      <c r="C114" s="8" t="inlineStr"/>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>Option A for safe harbor. Pay at least 90% of this year's tax to avoid penalty.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
@@ -1836,7 +2053,7 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>110% applies if prior-year AGI &gt; $150,000</t>
+          <t>Option B. If 2024 AGI &gt;$150K, you need 110% of 2024 tax, not 100%. Prior-year safe harbor is often easier to hit.</t>
         </is>
       </c>
     </row>
@@ -1850,7 +2067,11 @@
         <f>MIN($B$114, $B$115)</f>
         <v/>
       </c>
-      <c r="C116" s="8" t="inlineStr"/>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>You only need to hit the LOWER of Option A or B. Usually Option B (prior year) is easier.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
@@ -1862,7 +2083,11 @@
         <f>MAX(0, ($B$116-$B$106-$B$107)/$B$16)</f>
         <v/>
       </c>
-      <c r="C117" s="8" t="inlineStr"/>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Minimum extra withholding per check to avoid underpayment penalty. May be less than full break-even amount.</t>
+        </is>
+      </c>
       <c r="D117" s="16" t="n"/>
     </row>
     <row r="118" ht="6" customHeight="1">
@@ -1873,7 +2098,7 @@
     <row r="119" ht="40" customHeight="1">
       <c r="A119" s="18" t="inlineStr">
         <is>
-          <t>COMPARISON: paste the values from `twe estimate` output (or the web UI) into column D on the matching rows above. Differences &gt; $1 indicate a discrepancy to investigate.</t>
+          <t>COMPARISON: paste values from `twe estimate` (or the web UI) into column D on matching rows. Differences &gt; $1 indicate a discrepancy to investigate. See the 'How It Works' tab for explanations of each calculation step.</t>
         </is>
       </c>
     </row>
@@ -1885,4 +2110,478 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How the Estimator Computes Your Withholding</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Plain-English explanation of each section on the 'Verify 2025' sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>OVERVIEW</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>This sheet walks through how the Tax Withholding Estimator (TWE) calculates your recommended federal withholding per paycheck. Each section below matches a numbered section on the Verify 2025 sheet. Change the yellow input cells there and every formula updates automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>① INPUTS</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Filing status</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Controls which tax bracket table and standard deduction amount are used. The four options are: single, married_jointly, married_separately, head_of_household. The Verify 2025 sheet is pre-set to 'single' with 2025 single-filer constants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Standard deduction 2025</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Single: $15,000 | Married jointly: $30,000 | Head of household: $22,500 | Married separately: $15,000. Add $2,000 if single and age 65+ or blind (add $1,600 per qualifying person if married jointly).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Pay periods per year</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Weekly = 52 | Biweekly = 26 | Semimonthly = 24 | Monthly = 12. Your paystub should show pay period or check date — count how many times per year you receive a paycheck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Taxable wages this period</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>The gross wages that appear in Box 1 of your W-2 equivalent. This is NOT your gross pay — it is gross pay MINUS pre-tax deductions (401k, HSA, medical premiums, FSA, etc.). Your paystub may label this 'Federal Taxable' or 'Current Taxable Wages'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>② INCOME PROJECTION — how YTD is inferred</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Elapsed periods</t>
+        </is>
+      </c>
+      <c r="B11" s="21">
+        <f> periods_per_year − remaining_periods.
+Example: biweekly (26) with 14 remaining → 26 − 14 = 12 elapsed.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="104" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  YTD taxable wages — if you leave it at 0</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>The tool infers it as: elapsed_periods × taxable_wages_per_period.
+Example: 12 elapsed × $2,950/period = $35,400 inferred YTD wages.
+If you enter a non-zero value, the actual YTD figure from your paystub is used instead. Always prefer the real number from your paystub because it accounts for mid-year changes in pay rate or deductions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  YTD withholding — if you leave it at 0</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Same inference logic: elapsed_periods × withholding_per_period.
+Again, if your paystub shows a YTD federal tax withheld amount, enter that real number — it is more accurate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Projected wages</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f> YTD_wages_used + (remaining_periods × taxable_wages_per_period).
+This is the best estimate of what Box 1 of your W-2 will say.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>③ ADJUSTMENTS → AGI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
+    </row>
+    <row r="16" ht="118" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  What counts as an adjustment?</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Above-the-line deductions reduce income BEFORE the standard/itemized deduction is applied. Common ones:
+• Traditional IRA contribution (if deductible) — up to $7,000 ($8,000 age 50+)
+• HSA contribution (employee portion) — up to $4,300 single / $8,550 family
+• Student loan interest paid — up to $2,500
+• One-half of self-employment tax (computed automatically in Section ⑦)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  One-half SE tax approximation in Section ③</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Section ③ uses a quick approximation so AGI can be estimated early. Section ⑦ computes the exact SE tax. If you have SE income, confirm the exact half-SE deduction matches between the two sections — they should be within a few dollars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>④ DEDUCTION → TAXABLE INCOME</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="62" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Standard vs. itemized</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>The tool picks whichever is larger. If your itemized deductions (mortgage interest, state taxes up to $10K, charitable contributions, unreimbursed medical over 7.5% of AGI) exceed the standard deduction, enter your itemized total in the input cell. Otherwise leave it at 0 and the standard deduction applies automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Taxable income</t>
+        </is>
+      </c>
+      <c r="B20" s="21">
+        <f> AGI − deduction (standard or itemized, whichever is larger).
+This is the number the ordinary tax brackets are applied to, after the LTCG/qualified dividend portion is separated out.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>⑤ ORDINARY INCOME TAX — how brackets work</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="104" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LTCG / qualified dividends are separated first</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Long-term capital gains and qualified dividends get their own preferential rate (0/15/20%). They are removed from ordinary taxable income so the ordinary brackets apply only to wages, interest, short-term gains, etc.
+Preferential income = MIN(LTCG + qual_dividends, taxable_income)
+Ordinary TI = taxable_income − preferential_income</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="244" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bracket math (single, 2025)</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>The brackets are cumulative — each bracket only taxes the income WITHIN that range, not all income at the higher rate:
+  $0 – $11,925          → 10%  (max tax: $1,192.50)
+  $11,925 – $48,475      → 12%  (max additional: $4,386.00)
+  $48,475 – $103,350     → 22%  (max additional: $12,072.50)
+  $103,350 – $197,300    → 24%  (max additional: $22,548.00)
+  $197,300 – $250,525    → 32%  (max additional: $17,032.00)
+  $250,525 – $626,350    → 35%  (max additional: $131,538.75)
+  Over $626,350          → 37%
+The IFS formula on the Verify sheet encodes the cumulative amounts at each breakpoint so it only needs one lookup rather than stacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>⑥ CAPITAL GAINS TAX — 'stacking' explained</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n"/>
+    </row>
+    <row r="25" ht="216" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Why LTCG rates depend on ordinary income</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>The 0%/15%/20% LTCG rate thresholds apply to TOTAL taxable income (ordinary + preferential combined), not just the gains themselves. So if your ordinary income already uses up the 0% room, your gains are taxed at 15% even if they would otherwise fall below the threshold.
+Example (single 2025):
+  Ordinary TI = $40,000 → uses $40,000 of the $48,350 zero-rate room
+  Room remaining = $48,350 − $40,000 = $8,350
+  LTCG = $5,000 → first $8,350 of LTCG taxed at 0%, so all $5,000 = 0%
+  Ordinary TI = $50,000 → already exceeds $48,350, zero-rate room = $0
+  LTCG = $5,000 → all taxed at 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>⑦ SELF-EMPLOYMENT TAX</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n"/>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Why the 0.9235 factor?</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>As an employee, your employer pays half of FICA (SS + Medicare). Self-employed people pay both halves, but the IRS lets you deduct the employer-equivalent half. The 0.9235 factor (= 1 − 0.0765) approximates this: it reduces your net earnings to the amount that would be left after a hypothetical employer's 7.65% share is removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Social Security wage base</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>2025 SS wage base = $176,100. Only earnings up to this amount are subject to the 12.4% SS portion. Medicare (2.9%) has no cap. If your projected wages already exceed $176,100, none of your SE income faces SS tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  One-half SE tax deduction</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Half of your total SE tax (SS + Medicare) is deductible above the line, reducing AGI. Section ③ estimates this; Section ⑦ computes it exactly. If SE income is large, update the half-SE input in Section ③ to the exact value from Section ⑦ for a more accurate AGI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>⑧ ADDITIONAL MEDICARE TAX &amp; NIIT</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n"/>
+    </row>
+    <row r="31" ht="48" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Additional Medicare Tax (0.9%)</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Applies to wages/SE earnings over $200,000 (single), $250,000 (married jointly), $125,000 (married separately). Your employer withholds this automatically once your wages exceed $200K in a calendar year, but they do NOT know about your spouse's wages or SE income — you may owe more at filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Net Investment Income Tax — NIIT (3.8%)</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Applies to the LESSER of:
+  (a) net investment income (interest + dividends + capital gains), or
+  (b) AGI − $200,000 (single) / $250,000 (MFJ)
+If your AGI is below $200K, NIIT is $0 regardless of investment income.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>⑨ TAX LIABILITY</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n"/>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Order of credits</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>Nonrefundable credits (Child Tax Credit, education credits, etc.) reduce tax but cannot create a refund — they stop at $0 tax. Refundable credits (EITC, Additional Child Tax Credit) can produce a refund even if tax = $0. The tool applies nonrefundable credits first, then refundable credits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>⑩ WITHHOLDING RECOMMENDATION</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n"/>
+    </row>
+    <row r="36" ht="216" customHeight="1">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  How the per-paycheck number is calculated</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>1. Compute total liability (Section ⑨)
+2. Add target refund (usually $0 for break-even)
+3. Subtract everything already secured:
+   • YTD withholding from your paystub
+   • Estimated tax payments already made
+   • Spouse/other withholding
+4. Result = amount still needed from remaining paychecks
+5. Divide by remaining_periods → recommended per-paycheck withholding
+6. If that exceeds your normal withholding, the difference is what to
+   enter on Form W-4 line 4(c) as extra withholding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Target refund</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>Set to $0 to break even. A positive target refund (e.g. $500) means you want to over-withhold by that amount so you get a refund at filing. A negative target means you accept owing up to that amount at filing (only safe if within safe-harbor limits — see Section ⑪).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>⑪ SAFE HARBOR — penalty avoidance</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n"/>
+    </row>
+    <row r="39" ht="132" customHeight="1">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  What is safe harbor?</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>The IRS waives the underpayment penalty if you paid the lesser of:
+  (a) 90% of this year's tax liability, OR
+  (b) 100% of last year's tax (110% if last year's AGI exceeded $150,000)
+Safe harbor does NOT protect you from owing money — it just means no penalty on top of what you owe. The Section ⑪ row on the Verify sheet shows how much additional withholding per check is needed to hit this minimum, as an alternative to the full break-even recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  High-income rule (110%)</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>If your prior-year AGI was over $150,000 (single or married jointly), you must pay 110% of last year's tax (not 100%) to qualify for the prior-year safe harbor. Married filing separately threshold: $75,000. This is captured in the IFS formula in Section ⑪.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>